<commit_message>
Added file to file comparison feature.
</commit_message>
<xml_diff>
--- a/samples/oracle_hcm_source.xlsx
+++ b/samples/oracle_hcm_source.xlsx
@@ -418,154 +418,154 @@
     <t>GARCIA</t>
   </si>
   <si>
-    <t>22-SEP-1978</t>
-  </si>
-  <si>
-    <t>19-SEP-1981</t>
-  </si>
-  <si>
-    <t>26-MAY-1973</t>
-  </si>
-  <si>
-    <t>26-APR-1993</t>
-  </si>
-  <si>
-    <t>04-NOV-1984</t>
-  </si>
-  <si>
-    <t>08-JUN-1993</t>
-  </si>
-  <si>
-    <t>08-NOV-1990</t>
-  </si>
-  <si>
-    <t>14-FEB-1990</t>
-  </si>
-  <si>
-    <t>09-AUG-1972</t>
-  </si>
-  <si>
-    <t>21-MAR-1978</t>
-  </si>
-  <si>
-    <t>23-FEB-1990</t>
-  </si>
-  <si>
-    <t>22-JUL-1978</t>
-  </si>
-  <si>
-    <t>29-MAY-2016</t>
-  </si>
-  <si>
-    <t>29-MAR-1977</t>
-  </si>
-  <si>
-    <t>05-AUG-1992</t>
-  </si>
-  <si>
-    <t>06-SEP-1974</t>
-  </si>
-  <si>
-    <t>23-JAN-1988</t>
-  </si>
-  <si>
-    <t>27-JUL-1977</t>
-  </si>
-  <si>
-    <t>06-MAR-1971</t>
-  </si>
-  <si>
-    <t>15-JUL-1997</t>
-  </si>
-  <si>
-    <t>04-JUL-1973</t>
-  </si>
-  <si>
-    <t>12-MAY-1991</t>
-  </si>
-  <si>
-    <t>25-FEB-1994</t>
-  </si>
-  <si>
-    <t>17-JUN-1998</t>
-  </si>
-  <si>
-    <t>09-NOV-1983</t>
-  </si>
-  <si>
-    <t>29-JUN-1983</t>
-  </si>
-  <si>
-    <t>21-JUN-1983</t>
-  </si>
-  <si>
-    <t>05-OCT-1985</t>
+    <t>23-SEP-1978</t>
+  </si>
+  <si>
+    <t>20-SEP-1981</t>
+  </si>
+  <si>
+    <t>27-MAY-1973</t>
+  </si>
+  <si>
+    <t>27-APR-1993</t>
+  </si>
+  <si>
+    <t>05-NOV-1984</t>
+  </si>
+  <si>
+    <t>09-JUN-1993</t>
+  </si>
+  <si>
+    <t>09-NOV-1990</t>
+  </si>
+  <si>
+    <t>15-FEB-1990</t>
+  </si>
+  <si>
+    <t>10-AUG-1972</t>
   </si>
   <si>
     <t>22-MAR-1978</t>
   </si>
   <si>
-    <t>05-MAR-1998</t>
-  </si>
-  <si>
-    <t>22-FEB-1993</t>
-  </si>
-  <si>
-    <t>03-FEB-1983</t>
-  </si>
-  <si>
-    <t>27-JAN-1984</t>
-  </si>
-  <si>
-    <t>23-NOV-1971</t>
-  </si>
-  <si>
-    <t>12-JUL-1981</t>
-  </si>
-  <si>
-    <t>26-MAY-1981</t>
-  </si>
-  <si>
-    <t>02-MAR-1981</t>
-  </si>
-  <si>
-    <t>15-MAY-1993</t>
-  </si>
-  <si>
-    <t>19-JUL-1983</t>
-  </si>
-  <si>
-    <t>23-NOV-1992</t>
-  </si>
-  <si>
-    <t>21-APR-1970</t>
-  </si>
-  <si>
-    <t>14-SEP-1998</t>
-  </si>
-  <si>
-    <t>09-MAY-1985</t>
-  </si>
-  <si>
-    <t>02-AUG-1979</t>
-  </si>
-  <si>
-    <t>14-JUL-1992</t>
-  </si>
-  <si>
-    <t>14-APR-1980</t>
-  </si>
-  <si>
-    <t>17-NOV-1974</t>
-  </si>
-  <si>
-    <t>25-JUN-1992</t>
-  </si>
-  <si>
-    <t>22-MAR-1999</t>
-  </si>
-  <si>
-    <t>11-NOV-1993</t>
+    <t>24-FEB-1990</t>
+  </si>
+  <si>
+    <t>23-JUL-1978</t>
+  </si>
+  <si>
+    <t>30-MAY-2016</t>
+  </si>
+  <si>
+    <t>30-MAR-1977</t>
+  </si>
+  <si>
+    <t>06-AUG-1992</t>
+  </si>
+  <si>
+    <t>07-SEP-1974</t>
+  </si>
+  <si>
+    <t>24-JAN-1988</t>
+  </si>
+  <si>
+    <t>28-JUL-1977</t>
+  </si>
+  <si>
+    <t>07-MAR-1971</t>
+  </si>
+  <si>
+    <t>16-JUL-1997</t>
+  </si>
+  <si>
+    <t>05-JUL-1973</t>
+  </si>
+  <si>
+    <t>13-MAY-1991</t>
+  </si>
+  <si>
+    <t>26-FEB-1994</t>
+  </si>
+  <si>
+    <t>18-JUN-1998</t>
+  </si>
+  <si>
+    <t>10-NOV-1983</t>
+  </si>
+  <si>
+    <t>30-JUN-1983</t>
+  </si>
+  <si>
+    <t>22-JUN-1983</t>
+  </si>
+  <si>
+    <t>06-OCT-1985</t>
+  </si>
+  <si>
+    <t>23-MAR-1978</t>
+  </si>
+  <si>
+    <t>06-MAR-1998</t>
+  </si>
+  <si>
+    <t>23-FEB-1993</t>
+  </si>
+  <si>
+    <t>04-FEB-1983</t>
+  </si>
+  <si>
+    <t>28-JAN-1984</t>
+  </si>
+  <si>
+    <t>24-NOV-1971</t>
+  </si>
+  <si>
+    <t>13-JUL-1981</t>
+  </si>
+  <si>
+    <t>27-MAY-1981</t>
+  </si>
+  <si>
+    <t>03-MAR-1981</t>
+  </si>
+  <si>
+    <t>16-MAY-1993</t>
+  </si>
+  <si>
+    <t>20-JUL-1983</t>
+  </si>
+  <si>
+    <t>24-NOV-1992</t>
+  </si>
+  <si>
+    <t>22-APR-1970</t>
+  </si>
+  <si>
+    <t>15-SEP-1998</t>
+  </si>
+  <si>
+    <t>10-MAY-1985</t>
+  </si>
+  <si>
+    <t>03-AUG-1979</t>
+  </si>
+  <si>
+    <t>15-JUL-1992</t>
+  </si>
+  <si>
+    <t>15-APR-1980</t>
+  </si>
+  <si>
+    <t>18-NOV-1974</t>
+  </si>
+  <si>
+    <t>26-JUN-1992</t>
+  </si>
+  <si>
+    <t>23-MAR-1999</t>
+  </si>
+  <si>
+    <t>12-NOV-1993</t>
   </si>
   <si>
     <t>SANA.DAVIS@COMPANY.COM</t>
@@ -865,172 +865,172 @@
     <t>+1 (703) 275-1878</t>
   </si>
   <si>
-    <t>04-MAR-2025</t>
-  </si>
-  <si>
-    <t>07-NOV-2023</t>
-  </si>
-  <si>
-    <t>19-JUN-2022</t>
-  </si>
-  <si>
-    <t>23-NOV-2026</t>
-  </si>
-  <si>
-    <t>21-OCT-2018</t>
-  </si>
-  <si>
-    <t>10-SEP-2025</t>
-  </si>
-  <si>
-    <t>19-SEP-2024</t>
-  </si>
-  <si>
-    <t>14-APR-2019</t>
-  </si>
-  <si>
-    <t>04-SEP-2018</t>
-  </si>
-  <si>
-    <t>22-DEC-2022</t>
-  </si>
-  <si>
-    <t>15-NOV-2022</t>
-  </si>
-  <si>
-    <t>09-JUL-2019</t>
-  </si>
-  <si>
-    <t>28-SEP-2023</t>
-  </si>
-  <si>
-    <t>02-NOV-2024</t>
-  </si>
-  <si>
-    <t>29-DEC-2018</t>
-  </si>
-  <si>
-    <t>08-MAY-2021</t>
-  </si>
-  <si>
-    <t>10-DEC-2021</t>
-  </si>
-  <si>
-    <t>04-OCT-2025</t>
-  </si>
-  <si>
-    <t>30-OCT-2019</t>
-  </si>
-  <si>
-    <t>10-OCT-2022</t>
-  </si>
-  <si>
-    <t>05-DEC-2022</t>
-  </si>
-  <si>
-    <t>23-JUN-2022</t>
-  </si>
-  <si>
-    <t>21-MAY-2023</t>
-  </si>
-  <si>
-    <t>26-MAR-2022</t>
-  </si>
-  <si>
-    <t>02-MAY-2024</t>
-  </si>
-  <si>
-    <t>27-FEB-2021</t>
-  </si>
-  <si>
-    <t>22-APR-2020</t>
-  </si>
-  <si>
-    <t>09-JAN-2025</t>
-  </si>
-  <si>
-    <t>14-DEC-2022</t>
-  </si>
-  <si>
-    <t>05-MAR-2020</t>
-  </si>
-  <si>
-    <t>07-DEC-2018</t>
-  </si>
-  <si>
-    <t>03-JUL-2025</t>
-  </si>
-  <si>
-    <t>15-FEB-2025</t>
-  </si>
-  <si>
-    <t>11-MAY-2021</t>
-  </si>
-  <si>
-    <t>30-MAR-2023</t>
-  </si>
-  <si>
-    <t>01-SEP-2021</t>
-  </si>
-  <si>
-    <t>12-DEC-2021</t>
-  </si>
-  <si>
-    <t>29-JAN-2021</t>
-  </si>
-  <si>
-    <t>15-JUL-2022</t>
-  </si>
-  <si>
-    <t>21-DEC-2025</t>
-  </si>
-  <si>
-    <t>12-JUL-2019</t>
-  </si>
-  <si>
-    <t>05-FEB-2024</t>
-  </si>
-  <si>
-    <t>07-MAR-2026</t>
-  </si>
-  <si>
-    <t>08-FEB-2021</t>
-  </si>
-  <si>
-    <t>04-SEP-2022</t>
-  </si>
-  <si>
-    <t>17-AUG-2023</t>
-  </si>
-  <si>
-    <t>20-JUL-2021</t>
-  </si>
-  <si>
-    <t>04-MAR-2024</t>
+    <t>05-MAR-2025</t>
+  </si>
+  <si>
+    <t>08-NOV-2023</t>
+  </si>
+  <si>
+    <t>20-JUN-2022</t>
+  </si>
+  <si>
+    <t>24-NOV-2026</t>
+  </si>
+  <si>
+    <t>22-OCT-2018</t>
+  </si>
+  <si>
+    <t>11-SEP-2025</t>
+  </si>
+  <si>
+    <t>20-SEP-2024</t>
+  </si>
+  <si>
+    <t>15-APR-2019</t>
+  </si>
+  <si>
+    <t>05-SEP-2018</t>
+  </si>
+  <si>
+    <t>23-DEC-2022</t>
+  </si>
+  <si>
+    <t>16-NOV-2022</t>
+  </si>
+  <si>
+    <t>10-JUL-2019</t>
+  </si>
+  <si>
+    <t>29-SEP-2023</t>
+  </si>
+  <si>
+    <t>03-NOV-2024</t>
+  </si>
+  <si>
+    <t>30-DEC-2018</t>
+  </si>
+  <si>
+    <t>09-MAY-2021</t>
+  </si>
+  <si>
+    <t>11-DEC-2021</t>
+  </si>
+  <si>
+    <t>05-OCT-2025</t>
+  </si>
+  <si>
+    <t>31-OCT-2019</t>
+  </si>
+  <si>
+    <t>11-OCT-2022</t>
+  </si>
+  <si>
+    <t>06-DEC-2022</t>
+  </si>
+  <si>
+    <t>24-JUN-2022</t>
+  </si>
+  <si>
+    <t>22-MAY-2023</t>
+  </si>
+  <si>
+    <t>27-MAR-2022</t>
+  </si>
+  <si>
+    <t>03-MAY-2024</t>
+  </si>
+  <si>
+    <t>28-FEB-2021</t>
+  </si>
+  <si>
+    <t>23-APR-2020</t>
+  </si>
+  <si>
+    <t>10-JAN-2025</t>
+  </si>
+  <si>
+    <t>15-DEC-2022</t>
+  </si>
+  <si>
+    <t>06-MAR-2020</t>
+  </si>
+  <si>
+    <t>08-DEC-2018</t>
+  </si>
+  <si>
+    <t>04-JUL-2025</t>
+  </si>
+  <si>
+    <t>16-FEB-2025</t>
+  </si>
+  <si>
+    <t>12-MAY-2021</t>
   </si>
   <si>
     <t>31-MAR-2023</t>
   </si>
   <si>
-    <t>18-DEC-2020</t>
-  </si>
-  <si>
-    <t>03-JUN-2018</t>
-  </si>
-  <si>
-    <t>03-JUN-1996</t>
-  </si>
-  <si>
-    <t>23-MAY-2022</t>
-  </si>
-  <si>
-    <t>29-APR-2026</t>
-  </si>
-  <si>
-    <t>19-NOV-2025</t>
-  </si>
-  <si>
-    <t>01-APR-2026</t>
+    <t>02-SEP-2021</t>
+  </si>
+  <si>
+    <t>13-DEC-2021</t>
+  </si>
+  <si>
+    <t>30-JAN-2021</t>
+  </si>
+  <si>
+    <t>16-JUL-2022</t>
+  </si>
+  <si>
+    <t>22-DEC-2025</t>
+  </si>
+  <si>
+    <t>13-JUL-2019</t>
+  </si>
+  <si>
+    <t>06-FEB-2024</t>
+  </si>
+  <si>
+    <t>08-MAR-2026</t>
+  </si>
+  <si>
+    <t>09-FEB-2021</t>
+  </si>
+  <si>
+    <t>05-SEP-2022</t>
+  </si>
+  <si>
+    <t>18-AUG-2023</t>
+  </si>
+  <si>
+    <t>21-JUL-2021</t>
+  </si>
+  <si>
+    <t>05-MAR-2024</t>
+  </si>
+  <si>
+    <t>01-APR-2023</t>
+  </si>
+  <si>
+    <t>19-DEC-2020</t>
+  </si>
+  <si>
+    <t>04-JUN-2018</t>
+  </si>
+  <si>
+    <t>04-JUN-1996</t>
+  </si>
+  <si>
+    <t>24-MAY-2022</t>
+  </si>
+  <si>
+    <t>30-APR-2026</t>
+  </si>
+  <si>
+    <t>20-NOV-2025</t>
+  </si>
+  <si>
+    <t>02-APR-2026</t>
   </si>
   <si>
     <t>A</t>

</xml_diff>